<commit_message>
Initial workings on feedback for project_tracker_authentication
Signed-off-by: gabrielSe <gabriel.sewaldmoises@ucalgary.ca>
</commit_message>
<xml_diff>
--- a/Iteration_2/Echo_Review/Echo/Project_Tracker_Authentication.xlsx
+++ b/Iteration_2/Echo_Review/Echo/Project_Tracker_Authentication.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED82832-3F66-854C-A74E-FDD9ECE85B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3911365E-620E-493B-A8F0-AA046EDD3D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="23260" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project tracker" sheetId="1" r:id="rId1"/>
@@ -37,6 +37,111 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{BDD4D4E8-5032-4C8B-BD62-C975299853BD}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Suggestion: 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Consider having a new page tracking your meetings and what progress has been made up to that meeting</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{778808BB-D9CC-4425-A305-FDBEC2517FBC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">I don't see any type of structure, sequence, or any type of Diagrams/models for your coding tasks. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Have you spent time modelling how these methods should function?</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="0" shapeId="0" xr:uid="{5BE9B9AE-89D9-4AE3-A355-2808F9549311}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Your Tracker is not calculating your Estimated work hours automatically. </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Refer to previous versions of the tracker document to reinstate it</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{92BBBAC7-DDF3-4732-B9B1-B96B6EB51263}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Remember to assign your tasks to clear assignees. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>You can use the "Setup" page for more convenience</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="38">
   <si>
@@ -163,7 +268,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;Over/Under flag&quot;;&quot;&quot;;&quot;&quot;"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="3" tint="-0.499984740745262"/>
@@ -318,6 +423,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -711,7 +829,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -731,7 +849,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -795,7 +913,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -815,7 +933,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1492,28 +1610,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1">
     <tabColor theme="6"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="3" customWidth="1"/>
-    <col min="2" max="4" width="18.7109375" style="20" customWidth="1"/>
-    <col min="5" max="6" width="18.7109375" style="21" customWidth="1"/>
-    <col min="7" max="8" width="18.7109375" style="20" customWidth="1"/>
-    <col min="9" max="10" width="16.85546875" style="21" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" style="3" customWidth="1"/>
+    <col min="2" max="4" width="18.7265625" style="20" customWidth="1"/>
+    <col min="5" max="6" width="18.7265625" style="21" customWidth="1"/>
+    <col min="7" max="8" width="18.7265625" style="20" customWidth="1"/>
+    <col min="9" max="10" width="16.81640625" style="21" customWidth="1"/>
     <col min="11" max="12" width="16" style="20" customWidth="1"/>
-    <col min="13" max="13" width="20.42578125" style="20" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="4.140625" style="2" customWidth="1"/>
-    <col min="16" max="40" width="3.28515625" style="2" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="2"/>
+    <col min="13" max="13" width="20.453125" style="20" customWidth="1"/>
+    <col min="14" max="14" width="6.7265625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="4.1796875" style="2" customWidth="1"/>
+    <col min="16" max="40" width="3.26953125" style="2" customWidth="1"/>
+    <col min="41" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1529,7 +1647,7 @@
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>
     </row>
-    <row r="2" spans="1:14" s="5" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:14" s="5" customFormat="1" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="12" t="s">
         <v>0</v>
@@ -1551,7 +1669,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
     </row>
-    <row r="3" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1567,7 +1685,7 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
     </row>
-    <row r="4" spans="1:14" s="5" customFormat="1" ht="62" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:14" s="5" customFormat="1" ht="61.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="18" t="s">
         <v>2</v>
@@ -1607,7 +1725,7 @@
       </c>
       <c r="N4" s="11"/>
     </row>
-    <row r="5" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="19" t="s">
         <v>14</v>
@@ -1639,7 +1757,7 @@
       <c r="M5" s="19"/>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="19" t="s">
         <v>16</v>
@@ -1671,7 +1789,7 @@
       <c r="M6" s="19"/>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="19" t="s">
         <v>17</v>
@@ -1703,7 +1821,7 @@
       <c r="M7" s="19"/>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="19" t="s">
         <v>18</v>
@@ -1735,7 +1853,7 @@
       <c r="M8" s="19"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="19" t="s">
         <v>19</v>
@@ -1767,7 +1885,7 @@
       <c r="M9" s="19"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="19" t="s">
         <v>20</v>
@@ -1799,7 +1917,7 @@
       <c r="M10" s="19"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="19" t="s">
         <v>21</v>
@@ -1831,7 +1949,7 @@
       <c r="M11" s="19"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="19" t="s">
         <v>22</v>
@@ -1863,7 +1981,7 @@
       <c r="M12" s="19"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="19" t="s">
         <v>24</v>
@@ -1895,7 +2013,7 @@
       <c r="M13" s="19"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="27" t="s">
         <v>25</v>
@@ -1927,7 +2045,7 @@
       <c r="M14" s="27"/>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="27" t="s">
         <v>26</v>
       </c>
@@ -1957,7 +2075,7 @@
       </c>
       <c r="M15" s="27"/>
     </row>
-    <row r="16" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="27" t="s">
         <v>27</v>
       </c>
@@ -1987,7 +2105,7 @@
       </c>
       <c r="M16" s="27"/>
     </row>
-    <row r="17" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="27" t="s">
         <v>28</v>
       </c>
@@ -2017,7 +2135,7 @@
       </c>
       <c r="M17" s="27"/>
     </row>
-    <row r="18" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="27" t="s">
         <v>29</v>
       </c>
@@ -2047,7 +2165,7 @@
       </c>
       <c r="M18" s="27"/>
     </row>
-    <row r="19" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="27"/>
       <c r="C19" s="27"/>
       <c r="D19" s="27"/>
@@ -2067,7 +2185,7 @@
       </c>
       <c r="M19" s="27"/>
     </row>
-    <row r="20" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="27"/>
       <c r="C20" s="27"/>
       <c r="D20" s="27"/>
@@ -2087,7 +2205,7 @@
       </c>
       <c r="M20" s="27"/>
     </row>
-    <row r="21" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="27"/>
       <c r="C21" s="27"/>
       <c r="D21" s="27"/>
@@ -2107,7 +2225,7 @@
       </c>
       <c r="M21" s="27"/>
     </row>
-    <row r="22" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
       <c r="D22" s="27"/>
@@ -2127,7 +2245,7 @@
       </c>
       <c r="M22" s="27"/>
     </row>
-    <row r="23" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="27"/>
       <c r="C23" s="27"/>
       <c r="D23" s="27"/>
@@ -2147,7 +2265,7 @@
       </c>
       <c r="M23" s="27"/>
     </row>
-    <row r="24" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="27"/>
       <c r="C24" s="27"/>
       <c r="D24" s="27"/>
@@ -2167,7 +2285,7 @@
       </c>
       <c r="M24" s="27"/>
     </row>
-    <row r="25" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="27"/>
       <c r="C25" s="27"/>
       <c r="D25" s="27"/>
@@ -2187,7 +2305,7 @@
       </c>
       <c r="M25" s="27"/>
     </row>
-    <row r="26" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
       <c r="D26" s="27"/>
@@ -2207,7 +2325,7 @@
       </c>
       <c r="M26" s="27"/>
     </row>
-    <row r="27" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="27"/>
       <c r="C27" s="27"/>
       <c r="D27" s="27"/>
@@ -2227,7 +2345,7 @@
       </c>
       <c r="M27" s="27"/>
     </row>
-    <row r="28" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="27"/>
       <c r="C28" s="27"/>
       <c r="D28" s="27"/>
@@ -2247,7 +2365,7 @@
       </c>
       <c r="M28" s="27"/>
     </row>
-    <row r="29" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="27"/>
       <c r="C29" s="27"/>
       <c r="D29" s="27"/>
@@ -2267,7 +2385,7 @@
       </c>
       <c r="M29" s="27"/>
     </row>
-    <row r="30" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
       <c r="D30" s="27"/>
@@ -2287,7 +2405,7 @@
       </c>
       <c r="M30" s="27"/>
     </row>
-    <row r="31" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="27"/>
       <c r="C31" s="27"/>
       <c r="D31" s="27"/>
@@ -2307,7 +2425,7 @@
       </c>
       <c r="M31" s="27"/>
     </row>
-    <row r="32" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="27"/>
       <c r="C32" s="27"/>
       <c r="D32" s="27"/>
@@ -2327,7 +2445,7 @@
       </c>
       <c r="M32" s="27"/>
     </row>
-    <row r="33" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="27"/>
       <c r="C33" s="27"/>
       <c r="D33" s="27"/>
@@ -2347,7 +2465,7 @@
       </c>
       <c r="M33" s="27"/>
     </row>
-    <row r="34" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="27"/>
       <c r="C34" s="27"/>
       <c r="D34" s="27"/>
@@ -2367,7 +2485,7 @@
       </c>
       <c r="M34" s="27"/>
     </row>
-    <row r="35" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="27"/>
       <c r="C35" s="27"/>
       <c r="D35" s="27"/>
@@ -2387,7 +2505,7 @@
       </c>
       <c r="M35" s="27"/>
     </row>
-    <row r="36" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="27"/>
       <c r="C36" s="27"/>
       <c r="D36" s="27"/>
@@ -2407,7 +2525,7 @@
       </c>
       <c r="M36" s="27"/>
     </row>
-    <row r="37" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="27"/>
       <c r="C37" s="27"/>
       <c r="D37" s="27"/>
@@ -2427,7 +2545,7 @@
       </c>
       <c r="M37" s="27"/>
     </row>
-    <row r="38" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="27"/>
       <c r="C38" s="27"/>
       <c r="D38" s="27"/>
@@ -2447,7 +2565,7 @@
       </c>
       <c r="M38" s="27"/>
     </row>
-    <row r="39" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="27"/>
       <c r="C39" s="27"/>
       <c r="D39" s="27"/>
@@ -2504,8 +2622,9 @@
   <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2517,21 +2636,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="13" customWidth="1"/>
-    <col min="2" max="3" width="18.42578125" style="24" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" style="14" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" style="13" customWidth="1"/>
+    <col min="2" max="3" width="18.453125" style="24" customWidth="1"/>
+    <col min="4" max="4" width="6.7265625" style="14" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13"/>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
     </row>
-    <row r="2" spans="1:4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:4" customFormat="1" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13"/>
       <c r="B2" s="17" t="s">
         <v>30</v>
@@ -2539,13 +2658,13 @@
       <c r="C2" s="14"/>
       <c r="D2" s="14"/>
     </row>
-    <row r="3" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13"/>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
       <c r="D3" s="14"/>
     </row>
-    <row r="4" spans="1:4" customFormat="1" ht="62" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:4" customFormat="1" ht="61.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15"/>
       <c r="B4" s="23" t="s">
         <v>31</v>
@@ -2555,7 +2674,7 @@
       </c>
       <c r="D4" s="16"/>
     </row>
-    <row r="5" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
       <c r="B5" s="23" t="s">
         <v>15</v>
@@ -2565,7 +2684,7 @@
       </c>
       <c r="D5" s="14"/>
     </row>
-    <row r="6" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13"/>
       <c r="B6" s="23" t="s">
         <v>23</v>
@@ -2575,7 +2694,7 @@
       </c>
       <c r="D6" s="14"/>
     </row>
-    <row r="7" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
       <c r="B7" s="23"/>
       <c r="C7" s="23" t="s">
@@ -2583,7 +2702,7 @@
       </c>
       <c r="D7" s="14"/>
     </row>
-    <row r="8" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="B8" s="23"/>
       <c r="C8" s="23" t="s">
@@ -2591,7 +2710,7 @@
       </c>
       <c r="D8" s="14"/>
     </row>
-    <row r="9" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13"/>
       <c r="B9" s="23"/>
       <c r="C9" s="23" t="s">
@@ -2599,13 +2718,13 @@
       </c>
       <c r="D9" s="14"/>
     </row>
-    <row r="10" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13"/>
       <c r="B10" s="24"/>
       <c r="C10" s="24"/>
       <c r="D10" s="14"/>
     </row>
-    <row r="11" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="24"/>
       <c r="C11" s="24"/>
@@ -2628,15 +2747,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2948,7 +3058,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -2968,15 +3078,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D99023F8-0F96-4650-8DC3-63EE0BD6CB59}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2997,7 +3108,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3009,6 +3120,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>

<commit_message>
More in-depth comments on risks and time management
Signed-off-by: gabrielSe <gabriel.sewaldmoises@ucalgary.ca>
</commit_message>
<xml_diff>
--- a/Iteration_2/Echo_Review/Echo/Project_Tracker_Authentication.xlsx
+++ b/Iteration_2/Echo_Review/Echo/Project_Tracker_Authentication.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3911365E-620E-493B-A8F0-AA046EDD3D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F93C0D-0F61-483B-A0F5-C493E0545A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -114,6 +114,31 @@
         </r>
       </text>
     </comment>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{5D7D2C79-BA4B-408E-B34C-01E6B9A31EAC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">General Note: your tasks must have a timeline coherence. 
+Your authentication services are primordial for certain networking services.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Because you have multiple trackers, make sure your subteam overviewers have estimated dates follow time coherence. For example, you cannot test the final version of your matchmaking functionalities if your profile/authentication ones are not finalized beforehand</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="D5" authorId="0" shapeId="0" xr:uid="{92BBBAC7-DDF3-4732-B9B1-B96B6EB51263}">
       <text>
         <r>
@@ -135,6 +160,84 @@
             <family val="2"/>
           </rPr>
           <t>You can use the "Setup" page for more convenience</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H12" authorId="0" shapeId="0" xr:uid="{37453EB1-190C-4A00-9677-681AD5267F34}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Time Allocation:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> I suspect your Profile implementation will not be extremely complex and thus  your quick estimate (3 days) to get it done. Still, bear in mind that this task has a relatively shorter period in comparison to your other ones. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Consider extending it so that your assignee can conduct more specific and efficient tests</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F14" authorId="0" shapeId="0" xr:uid="{D58B5075-4DA9-415A-9DDE-A7CCE501BFD4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Potential Risk: </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>some of your tests extend until 1 week prior to the project's due date.</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Consider bringing forward your estimated start dates by a week so that your team can safely test your Authentication functionalities</t>
         </r>
       </text>
     </comment>
@@ -2747,6 +2850,35 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3058,36 +3190,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D99023F8-0F96-4650-8DC3-63EE0BD6CB59}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3108,26 +3231,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>

<commit_message>
Grammar corrections. Should be final version
Signed-off-by: gabrielSe <gabriel.sewaldmoises@ucalgary.ca>
</commit_message>
<xml_diff>
--- a/Iteration_2/Echo_Review/Echo/Project_Tracker_Authentication.xlsx
+++ b/Iteration_2/Echo_Review/Echo/Project_Tracker_Authentication.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F93C0D-0F61-483B-A0F5-C493E0545A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C9C5012-A568-4685-912B-3747F7F1FA06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -125,7 +125,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">General Note: your tasks must have a timeline coherence. 
-Your authentication services are primordial for certain networking services.
+Remember that your authentication services are primordial for certain networking services.
 </t>
         </r>
         <r>
@@ -237,7 +237,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Consider bringing forward your estimated start dates by a week so that your team can safely test your Authentication functionalities</t>
+Consider anticipating your estimated start dates by a week so that your team can safely test your Authentication functionalities</t>
         </r>
       </text>
     </comment>

</xml_diff>

<commit_message>
Finalized workings on project_tracker_authentication for Team Echo
</commit_message>
<xml_diff>
--- a/Iteration_2/Echo_Review/Echo/Project_Tracker_Authentication.xlsx
+++ b/Iteration_2/Echo_Review/Echo/Project_Tracker_Authentication.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED82832-3F66-854C-A74E-FDD9ECE85B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C9C5012-A568-4685-912B-3747F7F1FA06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="23260" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project tracker" sheetId="1" r:id="rId1"/>
@@ -37,6 +37,214 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{BDD4D4E8-5032-4C8B-BD62-C975299853BD}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Suggestion: 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Consider having a new page tracking your meetings and what progress has been made up to that meeting</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{778808BB-D9CC-4425-A305-FDBEC2517FBC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">I don't see any type of structure, sequence, or any type of Diagrams/models for your coding tasks. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Have you spent time modelling how these methods should function?</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="0" shapeId="0" xr:uid="{5BE9B9AE-89D9-4AE3-A355-2808F9549311}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Your Tracker is not calculating your Estimated work hours automatically. </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Refer to previous versions of the tracker document to reinstate it</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{5D7D2C79-BA4B-408E-B34C-01E6B9A31EAC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">General Note: your tasks must have a timeline coherence. 
+Remember that your authentication services are primordial for certain networking services.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Because you have multiple trackers, make sure your subteam overviewers have estimated dates follow time coherence. For example, you cannot test the final version of your matchmaking functionalities if your profile/authentication ones are not finalized beforehand</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{92BBBAC7-DDF3-4732-B9B1-B96B6EB51263}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Remember to assign your tasks to clear assignees. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>You can use the "Setup" page for more convenience</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H12" authorId="0" shapeId="0" xr:uid="{37453EB1-190C-4A00-9677-681AD5267F34}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Time Allocation:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> I suspect your Profile implementation will not be extremely complex and thus  your quick estimate (3 days) to get it done. Still, bear in mind that this task has a relatively shorter period in comparison to your other ones. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Consider extending it so that your assignee can conduct more specific and efficient tests</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F14" authorId="0" shapeId="0" xr:uid="{D58B5075-4DA9-415A-9DDE-A7CCE501BFD4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Potential Risk: </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>some of your tests extend until 1 week prior to the project's due date.</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Consider anticipating your estimated start dates by a week so that your team can safely test your Authentication functionalities</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="38">
   <si>
@@ -163,7 +371,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;Over/Under flag&quot;;&quot;&quot;;&quot;&quot;"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="3" tint="-0.499984740745262"/>
@@ -318,6 +526,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -711,7 +932,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -731,7 +952,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -795,7 +1016,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -815,7 +1036,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1492,28 +1713,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1">
     <tabColor theme="6"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="3" customWidth="1"/>
-    <col min="2" max="4" width="18.7109375" style="20" customWidth="1"/>
-    <col min="5" max="6" width="18.7109375" style="21" customWidth="1"/>
-    <col min="7" max="8" width="18.7109375" style="20" customWidth="1"/>
-    <col min="9" max="10" width="16.85546875" style="21" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" style="3" customWidth="1"/>
+    <col min="2" max="4" width="18.7265625" style="20" customWidth="1"/>
+    <col min="5" max="6" width="18.7265625" style="21" customWidth="1"/>
+    <col min="7" max="8" width="18.7265625" style="20" customWidth="1"/>
+    <col min="9" max="10" width="16.81640625" style="21" customWidth="1"/>
     <col min="11" max="12" width="16" style="20" customWidth="1"/>
-    <col min="13" max="13" width="20.42578125" style="20" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="4.140625" style="2" customWidth="1"/>
-    <col min="16" max="40" width="3.28515625" style="2" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="2"/>
+    <col min="13" max="13" width="20.453125" style="20" customWidth="1"/>
+    <col min="14" max="14" width="6.7265625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="4.1796875" style="2" customWidth="1"/>
+    <col min="16" max="40" width="3.26953125" style="2" customWidth="1"/>
+    <col min="41" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1529,7 +1750,7 @@
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>
     </row>
-    <row r="2" spans="1:14" s="5" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:14" s="5" customFormat="1" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="12" t="s">
         <v>0</v>
@@ -1551,7 +1772,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
     </row>
-    <row r="3" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1567,7 +1788,7 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
     </row>
-    <row r="4" spans="1:14" s="5" customFormat="1" ht="62" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:14" s="5" customFormat="1" ht="61.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="18" t="s">
         <v>2</v>
@@ -1607,7 +1828,7 @@
       </c>
       <c r="N4" s="11"/>
     </row>
-    <row r="5" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="19" t="s">
         <v>14</v>
@@ -1639,7 +1860,7 @@
       <c r="M5" s="19"/>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="19" t="s">
         <v>16</v>
@@ -1671,7 +1892,7 @@
       <c r="M6" s="19"/>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="19" t="s">
         <v>17</v>
@@ -1703,7 +1924,7 @@
       <c r="M7" s="19"/>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="19" t="s">
         <v>18</v>
@@ -1735,7 +1956,7 @@
       <c r="M8" s="19"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="19" t="s">
         <v>19</v>
@@ -1767,7 +1988,7 @@
       <c r="M9" s="19"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="19" t="s">
         <v>20</v>
@@ -1799,7 +2020,7 @@
       <c r="M10" s="19"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="19" t="s">
         <v>21</v>
@@ -1831,7 +2052,7 @@
       <c r="M11" s="19"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="19" t="s">
         <v>22</v>
@@ -1863,7 +2084,7 @@
       <c r="M12" s="19"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:14" s="5" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:14" s="5" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="19" t="s">
         <v>24</v>
@@ -1895,7 +2116,7 @@
       <c r="M13" s="19"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="27" t="s">
         <v>25</v>
@@ -1927,7 +2148,7 @@
       <c r="M14" s="27"/>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="27" t="s">
         <v>26</v>
       </c>
@@ -1957,7 +2178,7 @@
       </c>
       <c r="M15" s="27"/>
     </row>
-    <row r="16" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="27" t="s">
         <v>27</v>
       </c>
@@ -1987,7 +2208,7 @@
       </c>
       <c r="M16" s="27"/>
     </row>
-    <row r="17" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="27" t="s">
         <v>28</v>
       </c>
@@ -2017,7 +2238,7 @@
       </c>
       <c r="M17" s="27"/>
     </row>
-    <row r="18" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="27" t="s">
         <v>29</v>
       </c>
@@ -2047,7 +2268,7 @@
       </c>
       <c r="M18" s="27"/>
     </row>
-    <row r="19" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="27"/>
       <c r="C19" s="27"/>
       <c r="D19" s="27"/>
@@ -2067,7 +2288,7 @@
       </c>
       <c r="M19" s="27"/>
     </row>
-    <row r="20" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="27"/>
       <c r="C20" s="27"/>
       <c r="D20" s="27"/>
@@ -2087,7 +2308,7 @@
       </c>
       <c r="M20" s="27"/>
     </row>
-    <row r="21" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="27"/>
       <c r="C21" s="27"/>
       <c r="D21" s="27"/>
@@ -2107,7 +2328,7 @@
       </c>
       <c r="M21" s="27"/>
     </row>
-    <row r="22" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
       <c r="D22" s="27"/>
@@ -2127,7 +2348,7 @@
       </c>
       <c r="M22" s="27"/>
     </row>
-    <row r="23" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="27"/>
       <c r="C23" s="27"/>
       <c r="D23" s="27"/>
@@ -2147,7 +2368,7 @@
       </c>
       <c r="M23" s="27"/>
     </row>
-    <row r="24" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="27"/>
       <c r="C24" s="27"/>
       <c r="D24" s="27"/>
@@ -2167,7 +2388,7 @@
       </c>
       <c r="M24" s="27"/>
     </row>
-    <row r="25" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="27"/>
       <c r="C25" s="27"/>
       <c r="D25" s="27"/>
@@ -2187,7 +2408,7 @@
       </c>
       <c r="M25" s="27"/>
     </row>
-    <row r="26" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
       <c r="D26" s="27"/>
@@ -2207,7 +2428,7 @@
       </c>
       <c r="M26" s="27"/>
     </row>
-    <row r="27" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="27"/>
       <c r="C27" s="27"/>
       <c r="D27" s="27"/>
@@ -2227,7 +2448,7 @@
       </c>
       <c r="M27" s="27"/>
     </row>
-    <row r="28" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="27"/>
       <c r="C28" s="27"/>
       <c r="D28" s="27"/>
@@ -2247,7 +2468,7 @@
       </c>
       <c r="M28" s="27"/>
     </row>
-    <row r="29" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="27"/>
       <c r="C29" s="27"/>
       <c r="D29" s="27"/>
@@ -2267,7 +2488,7 @@
       </c>
       <c r="M29" s="27"/>
     </row>
-    <row r="30" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
       <c r="D30" s="27"/>
@@ -2287,7 +2508,7 @@
       </c>
       <c r="M30" s="27"/>
     </row>
-    <row r="31" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="27"/>
       <c r="C31" s="27"/>
       <c r="D31" s="27"/>
@@ -2307,7 +2528,7 @@
       </c>
       <c r="M31" s="27"/>
     </row>
-    <row r="32" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="27"/>
       <c r="C32" s="27"/>
       <c r="D32" s="27"/>
@@ -2327,7 +2548,7 @@
       </c>
       <c r="M32" s="27"/>
     </row>
-    <row r="33" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="27"/>
       <c r="C33" s="27"/>
       <c r="D33" s="27"/>
@@ -2347,7 +2568,7 @@
       </c>
       <c r="M33" s="27"/>
     </row>
-    <row r="34" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="27"/>
       <c r="C34" s="27"/>
       <c r="D34" s="27"/>
@@ -2367,7 +2588,7 @@
       </c>
       <c r="M34" s="27"/>
     </row>
-    <row r="35" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="27"/>
       <c r="C35" s="27"/>
       <c r="D35" s="27"/>
@@ -2387,7 +2608,7 @@
       </c>
       <c r="M35" s="27"/>
     </row>
-    <row r="36" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="27"/>
       <c r="C36" s="27"/>
       <c r="D36" s="27"/>
@@ -2407,7 +2628,7 @@
       </c>
       <c r="M36" s="27"/>
     </row>
-    <row r="37" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="27"/>
       <c r="C37" s="27"/>
       <c r="D37" s="27"/>
@@ -2427,7 +2648,7 @@
       </c>
       <c r="M37" s="27"/>
     </row>
-    <row r="38" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="27"/>
       <c r="C38" s="27"/>
       <c r="D38" s="27"/>
@@ -2447,7 +2668,7 @@
       </c>
       <c r="M38" s="27"/>
     </row>
-    <row r="39" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="27"/>
       <c r="C39" s="27"/>
       <c r="D39" s="27"/>
@@ -2504,8 +2725,9 @@
   <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2517,21 +2739,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="13" customWidth="1"/>
-    <col min="2" max="3" width="18.42578125" style="24" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" style="14" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" style="13" customWidth="1"/>
+    <col min="2" max="3" width="18.453125" style="24" customWidth="1"/>
+    <col min="4" max="4" width="6.7265625" style="14" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13"/>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
     </row>
-    <row r="2" spans="1:4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:4" customFormat="1" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13"/>
       <c r="B2" s="17" t="s">
         <v>30</v>
@@ -2539,13 +2761,13 @@
       <c r="C2" s="14"/>
       <c r="D2" s="14"/>
     </row>
-    <row r="3" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13"/>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
       <c r="D3" s="14"/>
     </row>
-    <row r="4" spans="1:4" customFormat="1" ht="62" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:4" customFormat="1" ht="61.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15"/>
       <c r="B4" s="23" t="s">
         <v>31</v>
@@ -2555,7 +2777,7 @@
       </c>
       <c r="D4" s="16"/>
     </row>
-    <row r="5" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
       <c r="B5" s="23" t="s">
         <v>15</v>
@@ -2565,7 +2787,7 @@
       </c>
       <c r="D5" s="14"/>
     </row>
-    <row r="6" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13"/>
       <c r="B6" s="23" t="s">
         <v>23</v>
@@ -2575,7 +2797,7 @@
       </c>
       <c r="D6" s="14"/>
     </row>
-    <row r="7" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
       <c r="B7" s="23"/>
       <c r="C7" s="23" t="s">
@@ -2583,7 +2805,7 @@
       </c>
       <c r="D7" s="14"/>
     </row>
-    <row r="8" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="B8" s="23"/>
       <c r="C8" s="23" t="s">
@@ -2591,7 +2813,7 @@
       </c>
       <c r="D8" s="14"/>
     </row>
-    <row r="9" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13"/>
       <c r="B9" s="23"/>
       <c r="C9" s="23" t="s">
@@ -2599,13 +2821,13 @@
       </c>
       <c r="D9" s="14"/>
     </row>
-    <row r="10" spans="1:4" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:4" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13"/>
       <c r="B10" s="24"/>
       <c r="C10" s="24"/>
       <c r="D10" s="14"/>
     </row>
-    <row r="11" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="24"/>
       <c r="C11" s="24"/>
@@ -2637,6 +2859,26 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2948,26 +3190,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
   <ds:schemaRefs>
@@ -2977,6 +3199,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D99023F8-0F96-4650-8DC3-63EE0BD6CB59}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2997,18 +3231,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>